<commit_message>
Apply revised rates across site, database and quotes; add Side Table 01 A1
Rate revision from GE Kochi Product Prices.xlsx (Sheet5): 38 of 41 catalog
items repriced. Sheet5 stays the single source of truth — the stale fallback
rate columns in Product_Database.xlsx (Rates sheet + per-theme Rate columns,
58 cells) were resynced to match so the fallback path cannot serve old prices.

Adds Side Table 01 A1 to Modern Times Master Bedroom (PNG optimized 4.12MB ->
0.57MB by update_site.py, original kept as .png.orig) and marks its placement
in the database.

Introduces client-facing quote workbooks for both residences, generated from
the same per-room selections the site publishes, with rates read live from
Sheet5 and amounts formula-linked so quantities stay editable.

Verified: all 69 line items reconcile across Sheet5 -> MasterSummary!U ->
Product_Database -> site HTML -> quote, 0 discrepancies.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Product_Database.xlsx
+++ b/Product_Database.xlsx
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>111000</v>
+        <v>117000</v>
       </c>
     </row>
     <row r="4">
@@ -763,13 +763,13 @@
           <t>Master Bedroom</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Master Bedroom</t>
         </is>
       </c>
       <c r="R5" t="n">
-        <v>20000</v>
+        <v>21000</v>
       </c>
     </row>
     <row r="6">
@@ -980,7 +980,7 @@
         </is>
       </c>
       <c r="R10" t="n">
-        <v>17000</v>
+        <v>19000</v>
       </c>
     </row>
     <row r="11">
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>21000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="12">
@@ -1074,7 +1074,7 @@
         </is>
       </c>
       <c r="R12" t="n">
-        <v>26000</v>
+        <v>27000</v>
       </c>
     </row>
     <row r="13">
@@ -1338,7 +1338,7 @@
         </is>
       </c>
       <c r="R18" t="n">
-        <v>72000</v>
+        <v>78000</v>
       </c>
     </row>
     <row r="19">
@@ -1472,7 +1472,7 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>37000</v>
+        <v>38000</v>
       </c>
     </row>
     <row r="22">
@@ -1608,7 +1608,7 @@
         </is>
       </c>
       <c r="R24" t="n">
-        <v>27000</v>
+        <v>29000</v>
       </c>
     </row>
     <row r="25">
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="R25" t="n">
-        <v>35000</v>
+        <v>36000</v>
       </c>
     </row>
     <row r="26" ht="22.8" customHeight="1">
@@ -1702,7 +1702,7 @@
         </is>
       </c>
       <c r="R26" t="n">
-        <v>37000</v>
+        <v>38000</v>
       </c>
     </row>
     <row r="27">
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="R28" t="n">
-        <v>10000</v>
+        <v>11000</v>
       </c>
     </row>
     <row r="29">
@@ -1963,7 +1963,7 @@
         </is>
       </c>
       <c r="R32" t="n">
-        <v>85000</v>
+        <v>88000</v>
       </c>
     </row>
     <row r="33">
@@ -2007,7 +2007,7 @@
         </is>
       </c>
       <c r="R33" t="n">
-        <v>82000</v>
+        <v>88000</v>
       </c>
     </row>
     <row r="34">
@@ -2333,7 +2333,7 @@
         </is>
       </c>
       <c r="R41" t="n">
-        <v>106000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="42">
@@ -2529,7 +2529,7 @@
         </is>
       </c>
       <c r="R46" t="n">
-        <v>51000</v>
+        <v>55000</v>
       </c>
     </row>
     <row r="47">
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="R47" t="n">
-        <v>141000</v>
+        <v>146000</v>
       </c>
     </row>
     <row r="48">
@@ -2623,7 +2623,7 @@
         </is>
       </c>
       <c r="R48" t="n">
-        <v>101000</v>
+        <v>106000</v>
       </c>
     </row>
     <row r="49">
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="R50" t="n">
-        <v>20000</v>
+        <v>22000</v>
       </c>
     </row>
     <row r="51">
@@ -2909,7 +2909,7 @@
         </is>
       </c>
       <c r="R55" t="n">
-        <v>149000</v>
+        <v>162000</v>
       </c>
     </row>
     <row r="56">
@@ -6340,7 +6340,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>17000</v>
+        <v>19000</v>
       </c>
     </row>
     <row r="3">
@@ -6350,7 +6350,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>21000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="4">
@@ -6360,7 +6360,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>26000</v>
+        <v>27000</v>
       </c>
     </row>
     <row r="5">
@@ -6370,7 +6370,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>100000</v>
+        <v>105000</v>
       </c>
     </row>
     <row r="6">
@@ -6380,7 +6380,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>111000</v>
+        <v>117000</v>
       </c>
     </row>
     <row r="7">
@@ -6390,7 +6390,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>141000</v>
+        <v>146000</v>
       </c>
     </row>
     <row r="8">
@@ -6400,7 +6400,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>98000</v>
+        <v>103000</v>
       </c>
     </row>
     <row r="9">
@@ -6410,7 +6410,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>24000</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="10">
@@ -6420,7 +6420,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>47000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="11">
@@ -6430,7 +6430,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>37000</v>
+        <v>38000</v>
       </c>
     </row>
     <row r="12">
@@ -6440,7 +6440,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>30000</v>
+        <v>32000</v>
       </c>
     </row>
     <row r="13">
@@ -6450,7 +6450,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>27000</v>
+        <v>29000</v>
       </c>
     </row>
     <row r="14">
@@ -6460,7 +6460,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>20000</v>
+        <v>22000</v>
       </c>
     </row>
     <row r="15">
@@ -6480,7 +6480,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>35000</v>
+        <v>36000</v>
       </c>
     </row>
     <row r="17">
@@ -6490,7 +6490,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>29000</v>
+        <v>31000</v>
       </c>
     </row>
     <row r="18">
@@ -6500,7 +6500,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>20000</v>
+        <v>21000</v>
       </c>
     </row>
     <row r="19">
@@ -6510,7 +6510,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>26000</v>
+        <v>27000</v>
       </c>
     </row>
     <row r="20">
@@ -6520,7 +6520,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>24000</v>
+        <v>26000</v>
       </c>
     </row>
     <row r="21">
@@ -6530,7 +6530,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>37000</v>
+        <v>38000</v>
       </c>
     </row>
     <row r="22">
@@ -6550,7 +6550,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>72000</v>
+        <v>78000</v>
       </c>
     </row>
     <row r="24">
@@ -6560,7 +6560,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>20000</v>
+        <v>21000</v>
       </c>
     </row>
     <row r="25">
@@ -6570,7 +6570,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>10000</v>
+        <v>11000</v>
       </c>
     </row>
     <row r="26">
@@ -6590,7 +6590,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>31000</v>
+        <v>33000</v>
       </c>
     </row>
     <row r="28">
@@ -6600,7 +6600,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>9000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="29">
@@ -6610,7 +6610,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>28000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="30">
@@ -6620,7 +6620,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>85000</v>
+        <v>88000</v>
       </c>
     </row>
     <row r="31">
@@ -6630,7 +6630,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>106000</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="32">
@@ -6640,7 +6640,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>101000</v>
+        <v>106000</v>
       </c>
     </row>
     <row r="33">
@@ -6650,7 +6650,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>82000</v>
+        <v>88000</v>
       </c>
     </row>
     <row r="34">
@@ -6660,7 +6660,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>54000</v>
+        <v>58000</v>
       </c>
     </row>
     <row r="35">
@@ -6670,7 +6670,7 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>82000</v>
+        <v>88000</v>
       </c>
     </row>
     <row r="36">
@@ -6680,7 +6680,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>44000</v>
+        <v>47000</v>
       </c>
     </row>
     <row r="37">
@@ -6690,7 +6690,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>51000</v>
+        <v>55000</v>
       </c>
     </row>
     <row r="38">
@@ -6700,7 +6700,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>77000</v>
+        <v>79000</v>
       </c>
     </row>
     <row r="39">
@@ -6710,7 +6710,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>65000</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="40">
@@ -6730,7 +6730,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>97000</v>
+        <v>101000</v>
       </c>
     </row>
     <row r="42">
@@ -6740,7 +6740,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>129000</v>
+        <v>135000</v>
       </c>
     </row>
     <row r="43">
@@ -6750,7 +6750,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>59000</v>
+        <v>64000</v>
       </c>
     </row>
     <row r="44">
@@ -6760,7 +6760,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>149000</v>
+        <v>162000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>